<commit_message>
Start of 2026 season, with Claude functions
</commit_message>
<xml_diff>
--- a/site/res/json/_Last-month-raceData.xlsx
+++ b/site/res/json/_Last-month-raceData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\git\frimleyFlyers\site\res\json\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B0E80D1-9CA0-4F8B-B596-E85DFE215AED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D015E1-483B-4DA8-9BE6-B4B6AE4E2AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23340" yWindow="3090" windowWidth="21600" windowHeight="11295" xr2:uid="{F8E35614-E497-4037-9098-C44996FE8116}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F8E35614-E497-4037-9098-C44996FE8116}"/>
   </bookViews>
   <sheets>
     <sheet name="b-raceData2024.json" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="74">
   <si>
     <t>Column1</t>
   </si>
@@ -61,9 +61,6 @@
     <t>Karen Peddle</t>
   </si>
   <si>
-    <t>Duncan Ball</t>
-  </si>
-  <si>
     <t>Christine Scally</t>
   </si>
   <si>
@@ -88,12 +85,6 @@
     <t>Jo Longmuir</t>
   </si>
   <si>
-    <t>Rebecca Williams</t>
-  </si>
-  <si>
-    <t>Charlotte Knight</t>
-  </si>
-  <si>
     <t>Jen Knight</t>
   </si>
   <si>
@@ -121,145 +112,136 @@
     <t>Susan Rodrigues</t>
   </si>
   <si>
-    <t xml:space="preserve">23:49	</t>
-  </si>
-  <si>
-    <t>Tom Churchill</t>
-  </si>
-  <si>
-    <t>Martin Gay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28:15	</t>
-  </si>
-  <si>
-    <t>Ben Gay</t>
-  </si>
-  <si>
-    <t>Frimley Lodge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:33	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">36:47	</t>
-  </si>
-  <si>
-    <t>Strathclyde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31:14	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29:30	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28:14	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:30	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24:47	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:31	</t>
-  </si>
-  <si>
     <t>Louise McIntosh</t>
   </si>
   <si>
-    <t>Lymington Woodside</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31:30	</t>
-  </si>
-  <si>
     <t>Karen Phillips</t>
   </si>
   <si>
     <t>Basingstoke</t>
   </si>
   <si>
-    <t xml:space="preserve">26:48	</t>
-  </si>
-  <si>
-    <t>Alan Bush</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20:33	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27:50	</t>
-  </si>
-  <si>
     <t>Harvey Ockrim</t>
   </si>
   <si>
-    <t xml:space="preserve">28:33	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28:29	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">36:05	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25:01	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:25	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">36:25	</t>
-  </si>
-  <si>
-    <t>Weymouth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29:07	</t>
-  </si>
-  <si>
     <t>Jodie Raynsford</t>
   </si>
   <si>
-    <t>Broadwater</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30:41	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">33:59	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">33:07	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">28:08	</t>
-  </si>
-  <si>
     <t>Andy Poulter</t>
   </si>
   <si>
-    <t xml:space="preserve">28:06	</t>
-  </si>
-  <si>
-    <t>Chris Peddle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">33:09	</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29:12	</t>
-  </si>
-  <si>
     <t>Simon Harvey</t>
   </si>
   <si>
-    <t xml:space="preserve">34:14	</t>
-  </si>
-  <si>
     <t>Column12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26:00	</t>
+  </si>
+  <si>
+    <t>Oli Peddle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:44	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:25	</t>
+  </si>
+  <si>
+    <t>Sarah Campbell-Foster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31:21	</t>
+  </si>
+  <si>
+    <t>Paul Bass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29:25	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29:41	</t>
+  </si>
+  <si>
+    <t>Simon Bass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29:44	</t>
+  </si>
+  <si>
+    <t>Coronation Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:50	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30:23	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25:34	</t>
+  </si>
+  <si>
+    <t>Phoebe Harvey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40:43	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32:59	</t>
+  </si>
+  <si>
+    <t>Brickfields Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34:37	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24:42	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30:17	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:24	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25:25	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24:18	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39:19	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31:32	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36:44	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36:19	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34:29	</t>
+  </si>
+  <si>
+    <t>Kirstie Stone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27:56	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">43:46	</t>
+  </si>
+  <si>
+    <t>Alasdair Nuttall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39:17	</t>
+  </si>
+  <si>
+    <t>David Peddle</t>
   </si>
 </sst>
 </file>
@@ -809,6 +791,14 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -824,14 +814,6 @@
         <name val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
       </font>
     </dxf>
   </dxfs>
@@ -854,11 +836,11 @@
     <sortCondition ref="E3:E36"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="6" xr3:uid="{2EE57549-C73C-457E-AC72-DDC94B55CE3B}" name="Column12" dataDxfId="0"/>
-    <tableColumn id="1" xr3:uid="{D3F63264-017A-4E07-B914-C5F98CA77055}" name="Column1" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{2EE57549-C73C-457E-AC72-DDC94B55CE3B}" name="Column12" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D3F63264-017A-4E07-B914-C5F98CA77055}" name="Column1" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{741C0D26-66B1-4900-9F9A-207388BA93A5}" name="Column2"/>
     <tableColumn id="3" xr3:uid="{AC85C6D5-0322-45AA-82DD-A19FD0112578}" name="Column3"/>
-    <tableColumn id="4" xr3:uid="{8711641C-9A00-4D46-9C48-CB28E1BCC94B}" name="Column4" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{8711641C-9A00-4D46-9C48-CB28E1BCC94B}" name="Column4" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{8727F302-2B57-4FB3-856C-2733213E68D8}" name="Column5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1185,15 +1167,15 @@
   <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22" style="2" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" style="2" customWidth="1"/>
     <col min="2" max="2" width="22" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1234,16 +1216,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E3" s="1">
-        <v>-0.158</v>
+        <v>-2.1899999999999999E-2</v>
       </c>
       <c r="F3" s="2">
         <v>26</v>
@@ -1254,16 +1236,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E4" s="1">
-        <v>-0.12520000000000001</v>
+        <v>-2.1499999999999998E-2</v>
       </c>
       <c r="F4" s="2">
         <v>22</v>
@@ -1274,19 +1256,19 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E5" s="1">
-        <v>-6.4000000000000001E-2</v>
+        <v>2.1499999999999998E-2</v>
       </c>
       <c r="F5" s="2">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1294,19 +1276,19 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E6" s="1">
-        <v>-5.0200000000000002E-2</v>
+        <v>3.5200000000000002E-2</v>
       </c>
       <c r="F6" s="2">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1314,19 +1296,19 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E7" s="1">
-        <v>-4.3200000000000002E-2</v>
+        <v>0.05</v>
       </c>
       <c r="F7" s="2">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1334,19 +1316,19 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E8" s="1">
-        <v>-3.5900000000000001E-2</v>
+        <v>5.1400000000000001E-2</v>
       </c>
       <c r="F8" s="2">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1354,19 +1336,19 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E9" s="1">
-        <v>-8.5000000000000006E-3</v>
+        <v>5.9400000000000001E-2</v>
       </c>
       <c r="F9" s="2">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1374,16 +1356,16 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E10" s="1">
-        <v>1.4999999999999999E-2</v>
+        <v>6.2399999999999997E-2</v>
       </c>
       <c r="F10" s="2">
         <v>4</v>
@@ -1394,16 +1376,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E11" s="1">
-        <v>1.5699999999999999E-2</v>
+        <v>6.4199999999999993E-2</v>
       </c>
       <c r="F11" s="2">
         <v>2</v>
@@ -1414,16 +1396,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="D12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E12" s="1">
-        <v>2.0500000000000001E-2</v>
+        <v>6.9000000000000006E-2</v>
       </c>
       <c r="F12" s="2">
         <v>1</v>
@@ -1434,16 +1416,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E13" s="1">
-        <v>2.1600000000000001E-2</v>
+        <v>6.9599999999999995E-2</v>
       </c>
       <c r="F13" s="2">
         <v>0</v>
@@ -1454,16 +1436,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D14" t="s">
         <v>55</v>
       </c>
       <c r="E14" s="1">
-        <v>2.41E-2</v>
+        <v>7.0300000000000001E-2</v>
       </c>
       <c r="F14" s="2">
         <v>0</v>
@@ -1474,16 +1456,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="C15" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="D15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E15" s="1">
-        <v>2.52E-2</v>
+        <v>7.5600000000000001E-2</v>
       </c>
       <c r="F15" s="2">
         <v>0</v>
@@ -1494,16 +1476,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
       <c r="E16" s="1">
-        <v>3.85E-2</v>
+        <v>8.9700000000000002E-2</v>
       </c>
       <c r="F16" s="2">
         <v>0</v>
@@ -1514,16 +1496,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="D17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E17" s="1">
-        <v>4.3200000000000002E-2</v>
+        <v>0.09</v>
       </c>
       <c r="F17" s="2">
         <v>0</v>
@@ -1534,16 +1516,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E18" s="1">
-        <v>6.1499999999999999E-2</v>
+        <v>9.2799999999999994E-2</v>
       </c>
       <c r="F18" s="2">
         <v>0</v>
@@ -1554,16 +1536,16 @@
         <v>17</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E19" s="1">
-        <v>6.2300000000000001E-2</v>
+        <v>9.4E-2</v>
       </c>
       <c r="F19" s="2">
         <v>0</v>
@@ -1574,16 +1556,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D20" t="s">
         <v>61</v>
       </c>
       <c r="E20" s="1">
-        <v>6.4500000000000002E-2</v>
+        <v>0.1019</v>
       </c>
       <c r="F20" s="2">
         <v>0</v>
@@ -1594,16 +1576,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D21" t="s">
         <v>62</v>
       </c>
       <c r="E21" s="1">
-        <v>7.3400000000000007E-2</v>
+        <v>0.10199999999999999</v>
       </c>
       <c r="F21" s="2">
         <v>0</v>
@@ -1614,16 +1596,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="C22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D22" t="s">
         <v>63</v>
       </c>
       <c r="E22" s="1">
-        <v>8.2199999999999995E-2</v>
+        <v>0.1133</v>
       </c>
       <c r="F22" s="2">
         <v>0</v>
@@ -1634,16 +1616,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="C23" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" t="s">
         <v>64</v>
       </c>
-      <c r="D23" t="s">
-        <v>65</v>
-      </c>
       <c r="E23" s="1">
-        <v>8.7800000000000003E-2</v>
+        <v>0.12089999999999999</v>
       </c>
       <c r="F23" s="2">
         <v>0</v>
@@ -1654,16 +1636,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="D24" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E24" s="1">
-        <v>9.5799999999999996E-2</v>
+        <v>0.13900000000000001</v>
       </c>
       <c r="F24" s="2">
         <v>0</v>
@@ -1674,16 +1656,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D25" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E25" s="1">
-        <v>0.13089999999999999</v>
+        <v>0.1628</v>
       </c>
       <c r="F25" s="2">
         <v>0</v>
@@ -1697,13 +1679,13 @@
         <v>13</v>
       </c>
       <c r="C26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D26" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E26" s="1">
-        <v>0.17430000000000001</v>
+        <v>0.2301</v>
       </c>
       <c r="F26" s="2">
         <v>0</v>
@@ -1714,16 +1696,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="C27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D27" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="E27" s="1">
-        <v>0.24299999999999999</v>
+        <v>0.2414</v>
       </c>
       <c r="F27" s="2">
         <v>0</v>
@@ -1734,16 +1716,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="C28" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="D28" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E28" s="1">
-        <v>0.26479999999999998</v>
+        <v>0.28129999999999999</v>
       </c>
       <c r="F28" s="2">
         <v>0</v>
@@ -1754,16 +1736,16 @@
         <v>27</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="C29" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D29" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E29" s="1">
-        <v>0.32690000000000002</v>
+        <v>0.52139999999999997</v>
       </c>
       <c r="F29" s="2">
         <v>0</v>
@@ -1774,16 +1756,16 @@
         <v>28</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="C30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D30" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E30" s="1">
-        <v>0.35499999999999998</v>
+        <v>0.54759999999999998</v>
       </c>
       <c r="F30" s="2">
         <v>0</v>
@@ -1794,16 +1776,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D31" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="E31" s="1">
-        <v>0.56910000000000005</v>
+        <v>0.74980000000000002</v>
       </c>
       <c r="F31" s="2">
         <v>0</v>
@@ -1814,13 +1796,13 @@
         <v>30</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D32" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E32" s="1">
         <v>0.23319999999999999</v>
@@ -1834,13 +1816,13 @@
         <v>31</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C33" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D33" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E33" s="1">
         <v>0.28539999999999999</v>

</xml_diff>